<commit_message>
adding debug for tests
</commit_message>
<xml_diff>
--- a/default_sample_pages.xlsx
+++ b/default_sample_pages.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA518B6A-3255-4165-B3B6-8034D737E5E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648"/>
+    <workbookView xWindow="2055" yWindow="2670" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="webpage" sheetId="1" r:id="rId1"/>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Webbsida</t>
   </si>
@@ -31,12 +32,18 @@
   </si>
   <si>
     <t>Startsida</t>
+  </si>
+  <si>
+    <t>https://github.com</t>
+  </si>
+  <si>
+    <t>Github</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -358,15 +365,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="101.77734375" customWidth="1"/>
+    <col min="1" max="1" width="101.7109375" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -374,17 +381,26 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="A3" r:id="rId2" xr:uid="{21901C41-4832-4789-94F4-B146A5AD77B1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>